<commit_message>
Updating the base path
</commit_message>
<xml_diff>
--- a/server/data/users/subbareddy.xlsx
+++ b/server/data/users/subbareddy.xlsx
@@ -437,7 +437,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -479,15 +479,35 @@
         <v>2026-01-30T15:12:39.313Z</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-01-30T15:12:59.592Z</v>
+        <v>2026-01-30T16:14:53.851Z</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>1769789671844</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Learning python</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Complete the course with in next 30 days</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-01-30T16:14:31.844Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-01-30T16:14:31.844Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>